<commit_message>
Almost working on Python 3 without GPU
</commit_message>
<xml_diff>
--- a/history_matching/example/iter1/Cuts/RadiusShouldBe15/history_matching_config.xlsx
+++ b/history_matching/example/iter1/Cuts/RadiusShouldBe15/history_matching_config.xlsx
@@ -2,6 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
     <workbookView activeTab="0"/>
   </bookViews>
@@ -17,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="80">
   <si>
     <t>Parameter</t>
   </si>
@@ -67,136 +68,181 @@
     <t>Train</t>
   </si>
   <si>
-    <t>Data_20170712_102507.000000</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000001</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000002</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000003</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000004</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000005</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000006</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000007</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000008</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000009</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000010</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000011</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000012</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000013</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000014</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000015</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000016</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000017</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000018</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000019</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000020</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000021</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000022</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000023</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000024</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000025</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000026</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000027</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000028</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000029</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000030</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000031</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000032</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000033</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000034</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000035</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000036</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000037</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000038</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000039</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000040</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000041</t>
-  </si>
-  <si>
-    <t>Data_20170712_102507.000042</t>
+    <t>Data_20180119_074303.000000</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000001</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000002</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000003</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000004</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000005</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000006</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000007</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000008</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000009</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000010</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000011</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000012</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000013</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000014</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000015</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000016</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000017</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000018</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000019</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000020</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000021</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000022</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000023</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000024</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000025</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000026</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000027</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000028</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000029</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000030</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000031</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000032</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000033</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000034</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000035</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000036</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000037</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000038</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000039</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000040</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000041</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000042</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000043</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000044</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000045</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000046</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000047</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000048</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000049</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000050</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000051</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000052</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000053</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000054</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000055</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000056</t>
+  </si>
+  <si>
+    <t>Data_20180119_074303.000057</t>
   </si>
   <si>
     <t>Sim_Id</t>
@@ -638,7 +684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F44"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
@@ -669,10 +715,10 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>-18.04118948177776</v>
+        <v>2.186099688264044</v>
       </c>
       <c r="D2" t="n">
-        <v>-11.64358846342563</v>
+        <v>-2.139445702561019</v>
       </c>
       <c r="E2" t="s">
         <v>17</v>
@@ -689,10 +735,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1.824148924904549</v>
+        <v>24.07984869323391</v>
       </c>
       <c r="D3" t="n">
-        <v>-16.24289861220373</v>
+        <v>-11.58956938733648</v>
       </c>
       <c r="E3" t="s">
         <v>17</v>
@@ -709,10 +755,10 @@
         <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>0.5685187880030469</v>
+        <v>-9.016405488666004</v>
       </c>
       <c r="D4" t="n">
-        <v>-17.79115785323854</v>
+        <v>-4.823317184306902</v>
       </c>
       <c r="E4" t="s">
         <v>17</v>
@@ -729,10 +775,10 @@
         <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>-5.057121594267954</v>
+        <v>4.859916288097089</v>
       </c>
       <c r="D5" t="n">
-        <v>-7.504572336221827</v>
+        <v>-31.32942135452733</v>
       </c>
       <c r="E5" t="s">
         <v>17</v>
@@ -749,10 +795,10 @@
         <v>4</v>
       </c>
       <c r="C6" t="n">
-        <v>-13.35251836315878</v>
+        <v>-16.02079393798419</v>
       </c>
       <c r="D6" t="n">
-        <v>15.78123281001729</v>
+        <v>-18.75135171052559</v>
       </c>
       <c r="E6" t="s">
         <v>17</v>
@@ -769,10 +815,10 @@
         <v>5</v>
       </c>
       <c r="C7" t="n">
-        <v>16.55353419180717</v>
+        <v>-22.21519901616071</v>
       </c>
       <c r="D7" t="n">
-        <v>10.86653090602863</v>
+        <v>19.67113524689151</v>
       </c>
       <c r="E7" t="s">
         <v>17</v>
@@ -789,10 +835,10 @@
         <v>6</v>
       </c>
       <c r="C8" t="n">
-        <v>2.96271503522054</v>
+        <v>14.71013225950182</v>
       </c>
       <c r="D8" t="n">
-        <v>5.913511551678141</v>
+        <v>-26.57688483605933</v>
       </c>
       <c r="E8" t="s">
         <v>17</v>
@@ -809,10 +855,10 @@
         <v>7</v>
       </c>
       <c r="C9" t="n">
-        <v>-16.53731150211988</v>
+        <v>-13.50780455188965</v>
       </c>
       <c r="D9" t="n">
-        <v>-18.64175006945499</v>
+        <v>-23.35173533077449</v>
       </c>
       <c r="E9" t="s">
         <v>17</v>
@@ -829,10 +875,10 @@
         <v>8</v>
       </c>
       <c r="C10" t="n">
-        <v>21.07190327309267</v>
+        <v>23.73451069352058</v>
       </c>
       <c r="D10" t="n">
-        <v>-7.579856232544273</v>
+        <v>5.534927670994279</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
@@ -849,10 +895,10 @@
         <v>9</v>
       </c>
       <c r="C11" t="n">
-        <v>1.920101219265611</v>
+        <v>-24.53380220870584</v>
       </c>
       <c r="D11" t="n">
-        <v>4.725526362327059</v>
+        <v>12.12810024526132</v>
       </c>
       <c r="E11" t="s">
         <v>17</v>
@@ -869,10 +915,10 @@
         <v>10</v>
       </c>
       <c r="C12" t="n">
-        <v>12.75674007460906</v>
+        <v>2.314465242766595</v>
       </c>
       <c r="D12" t="n">
-        <v>-8.815619801961887</v>
+        <v>8.694287936571882</v>
       </c>
       <c r="E12" t="s">
         <v>17</v>
@@ -889,10 +935,10 @@
         <v>11</v>
       </c>
       <c r="C13" t="n">
-        <v>-4.249593944633105</v>
+        <v>7.965501321120925</v>
       </c>
       <c r="D13" t="n">
-        <v>-15.37958019574265</v>
+        <v>-3.585598447696029</v>
       </c>
       <c r="E13" t="s">
         <v>17</v>
@@ -909,10 +955,10 @@
         <v>12</v>
       </c>
       <c r="C14" t="n">
-        <v>-21.86458171310274</v>
+        <v>-4.303288666319887</v>
       </c>
       <c r="D14" t="n">
-        <v>1.847808520566005</v>
+        <v>-20.87979074122815</v>
       </c>
       <c r="E14" t="s">
         <v>17</v>
@@ -929,10 +975,10 @@
         <v>13</v>
       </c>
       <c r="C15" t="n">
-        <v>-5.571714476901889</v>
+        <v>-8.9394739177012</v>
       </c>
       <c r="D15" t="n">
-        <v>24.17223276508321</v>
+        <v>33.20049266139981</v>
       </c>
       <c r="E15" t="s">
         <v>17</v>
@@ -949,10 +995,10 @@
         <v>14</v>
       </c>
       <c r="C16" t="n">
-        <v>-6.004526048560841</v>
+        <v>-0.08419433195268056</v>
       </c>
       <c r="D16" t="n">
-        <v>5.15883422605927</v>
+        <v>-30.95110736126681</v>
       </c>
       <c r="E16" t="s">
         <v>17</v>
@@ -969,10 +1015,10 @@
         <v>15</v>
       </c>
       <c r="C17" t="n">
-        <v>5.661716124110107</v>
+        <v>19.79603406496537</v>
       </c>
       <c r="D17" t="n">
-        <v>20.47606774644855</v>
+        <v>-6.700193283887272</v>
       </c>
       <c r="E17" t="s">
         <v>17</v>
@@ -989,10 +1035,10 @@
         <v>16</v>
       </c>
       <c r="C18" t="n">
-        <v>-10.92591156707768</v>
+        <v>-5.111771209066959</v>
       </c>
       <c r="D18" t="n">
-        <v>-0.8490017077678118</v>
+        <v>26.44239633506925</v>
       </c>
       <c r="E18" t="s">
         <v>17</v>
@@ -1009,10 +1055,10 @@
         <v>17</v>
       </c>
       <c r="C19" t="n">
-        <v>-4.590785578506953</v>
+        <v>-7.980370715859571</v>
       </c>
       <c r="D19" t="n">
-        <v>21.75514286552172</v>
+        <v>0.1087881473155221</v>
       </c>
       <c r="E19" t="s">
         <v>17</v>
@@ -1029,10 +1075,10 @@
         <v>18</v>
       </c>
       <c r="C20" t="n">
-        <v>11.55567018211899</v>
+        <v>20.24622118548824</v>
       </c>
       <c r="D20" t="n">
-        <v>3.266395746393158</v>
+        <v>-9.801395121028833</v>
       </c>
       <c r="E20" t="s">
         <v>17</v>
@@ -1049,10 +1095,10 @@
         <v>19</v>
       </c>
       <c r="C21" t="n">
-        <v>-30.99786334712302</v>
+        <v>6.748994980594944</v>
       </c>
       <c r="D21" t="n">
-        <v>1.245475460999799</v>
+        <v>-25.20939250478221</v>
       </c>
       <c r="E21" t="s">
         <v>17</v>
@@ -1069,10 +1115,10 @@
         <v>20</v>
       </c>
       <c r="C22" t="n">
-        <v>-25.28666245629316</v>
+        <v>-18.64576216183469</v>
       </c>
       <c r="D22" t="n">
-        <v>-10.31378029957536</v>
+        <v>-6.306020405177777</v>
       </c>
       <c r="E22" t="s">
         <v>17</v>
@@ -1089,10 +1135,10 @@
         <v>21</v>
       </c>
       <c r="C23" t="n">
-        <v>4.960357405121407</v>
+        <v>27.08979516205517</v>
       </c>
       <c r="D23" t="n">
-        <v>-20.29431573214625</v>
+        <v>-4.277371908924778</v>
       </c>
       <c r="E23" t="s">
         <v>17</v>
@@ -1109,10 +1155,10 @@
         <v>22</v>
       </c>
       <c r="C24" t="n">
-        <v>-1.12895076751893</v>
+        <v>-12.28982422068739</v>
       </c>
       <c r="D24" t="n">
-        <v>12.58552814364026</v>
+        <v>-2.942749773635683</v>
       </c>
       <c r="E24" t="s">
         <v>17</v>
@@ -1129,10 +1175,10 @@
         <v>23</v>
       </c>
       <c r="C25" t="n">
-        <v>-17.47176797706838</v>
+        <v>15.44367982075539</v>
       </c>
       <c r="D25" t="n">
-        <v>8.966087380030771</v>
+        <v>-12.56306782461934</v>
       </c>
       <c r="E25" t="s">
         <v>17</v>
@@ -1149,10 +1195,10 @@
         <v>24</v>
       </c>
       <c r="C26" t="n">
-        <v>-18.42129338948475</v>
+        <v>13.39850066047773</v>
       </c>
       <c r="D26" t="n">
-        <v>-1.476471144587819</v>
+        <v>11.78005320981035</v>
       </c>
       <c r="E26" t="s">
         <v>17</v>
@@ -1169,10 +1215,10 @@
         <v>25</v>
       </c>
       <c r="C27" t="n">
-        <v>6.591193711193156</v>
+        <v>-12.09171877772787</v>
       </c>
       <c r="D27" t="n">
-        <v>2.871834386803542</v>
+        <v>18.29232783467762</v>
       </c>
       <c r="E27" t="s">
         <v>17</v>
@@ -1189,10 +1235,10 @@
         <v>26</v>
       </c>
       <c r="C28" t="n">
-        <v>6.060258268142746</v>
+        <v>-21.07737516515695</v>
       </c>
       <c r="D28" t="n">
-        <v>8.470437825337228</v>
+        <v>-21.73273860322199</v>
       </c>
       <c r="E28" t="s">
         <v>17</v>
@@ -1209,10 +1255,10 @@
         <v>27</v>
       </c>
       <c r="C29" t="n">
-        <v>15.61652563484574</v>
+        <v>11.41422634931679</v>
       </c>
       <c r="D29" t="n">
-        <v>7.58037840049748</v>
+        <v>27.31241380752315</v>
       </c>
       <c r="E29" t="s">
         <v>17</v>
@@ -1229,10 +1275,10 @@
         <v>28</v>
       </c>
       <c r="C30" t="n">
-        <v>-9.693723687364702</v>
+        <v>1.632564786905078</v>
       </c>
       <c r="D30" t="n">
-        <v>-6.147619648382715</v>
+        <v>-1.693978941922325</v>
       </c>
       <c r="E30" t="s">
         <v>17</v>
@@ -1249,10 +1295,10 @@
         <v>29</v>
       </c>
       <c r="C31" t="n">
-        <v>14.34476951603071</v>
+        <v>-10.29776502369423</v>
       </c>
       <c r="D31" t="n">
-        <v>-0.5447391675731552</v>
+        <v>7.463092368956055</v>
       </c>
       <c r="E31" t="s">
         <v>17</v>
@@ -1269,10 +1315,10 @@
         <v>30</v>
       </c>
       <c r="C32" t="n">
-        <v>-0.9307075704026033</v>
+        <v>7.591842758822531</v>
       </c>
       <c r="D32" t="n">
-        <v>9.753552886461975</v>
+        <v>-5.482376897994327</v>
       </c>
       <c r="E32" t="s">
         <v>17</v>
@@ -1289,16 +1335,16 @@
         <v>31</v>
       </c>
       <c r="C33" t="n">
-        <v>-7.898153762611877</v>
+        <v>4.924640630203903</v>
       </c>
       <c r="D33" t="n">
-        <v>-11.98075745092109</v>
+        <v>6.119574885302598</v>
       </c>
       <c r="E33" t="s">
         <v>17</v>
       </c>
       <c r="F33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -1309,16 +1355,16 @@
         <v>32</v>
       </c>
       <c r="C34" t="n">
-        <v>-24.52284498465529</v>
+        <v>-6.206197874611312</v>
       </c>
       <c r="D34" t="n">
-        <v>-1.979899562656556</v>
+        <v>22.31628019576578</v>
       </c>
       <c r="E34" t="s">
         <v>17</v>
       </c>
       <c r="F34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -1329,16 +1375,16 @@
         <v>33</v>
       </c>
       <c r="C35" t="n">
-        <v>4.177455311109782</v>
+        <v>-9.57679161945309</v>
       </c>
       <c r="D35" t="n">
-        <v>13.73693115827579</v>
+        <v>14.04040503195403</v>
       </c>
       <c r="E35" t="s">
         <v>17</v>
       </c>
       <c r="F35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -1349,16 +1395,16 @@
         <v>34</v>
       </c>
       <c r="C36" t="n">
-        <v>6.353546242975462</v>
+        <v>-11.22740362589908</v>
       </c>
       <c r="D36" t="n">
-        <v>-16.18135742091141</v>
+        <v>-9.231346303046408</v>
       </c>
       <c r="E36" t="s">
         <v>17</v>
       </c>
       <c r="F36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -1369,16 +1415,16 @@
         <v>35</v>
       </c>
       <c r="C37" t="n">
-        <v>5.207803852178216</v>
+        <v>5.996932756823611</v>
       </c>
       <c r="D37" t="n">
-        <v>17.0070014045056</v>
+        <v>-13.79653451799263</v>
       </c>
       <c r="E37" t="s">
         <v>17</v>
       </c>
       <c r="F37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -1389,16 +1435,16 @@
         <v>36</v>
       </c>
       <c r="C38" t="n">
-        <v>14.45776138904563</v>
+        <v>19.21089343106291</v>
       </c>
       <c r="D38" t="n">
-        <v>18.46544097256609</v>
+        <v>-0.8386006665221544</v>
       </c>
       <c r="E38" t="s">
         <v>17</v>
       </c>
       <c r="F38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -1409,16 +1455,16 @@
         <v>37</v>
       </c>
       <c r="C39" t="n">
-        <v>0.9723046034035718</v>
+        <v>-23.5748263108685</v>
       </c>
       <c r="D39" t="n">
-        <v>-14.03956635398707</v>
+        <v>-11.54109296391725</v>
       </c>
       <c r="E39" t="s">
         <v>17</v>
       </c>
       <c r="F39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -1429,16 +1475,16 @@
         <v>38</v>
       </c>
       <c r="C40" t="n">
-        <v>-13.63797246068165</v>
+        <v>-12.75215359731575</v>
       </c>
       <c r="D40" t="n">
-        <v>-19.26519083757022</v>
+        <v>25.83285277671557</v>
       </c>
       <c r="E40" t="s">
         <v>17</v>
       </c>
       <c r="F40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -1449,16 +1495,16 @@
         <v>39</v>
       </c>
       <c r="C41" t="n">
-        <v>2.772618375806935</v>
+        <v>-16.35321082151363</v>
       </c>
       <c r="D41" t="n">
-        <v>9.375532043181707</v>
+        <v>-1.056625987281194</v>
       </c>
       <c r="E41" t="s">
         <v>17</v>
       </c>
       <c r="F41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -1469,16 +1515,16 @@
         <v>40</v>
       </c>
       <c r="C42" t="n">
-        <v>10.43538390339322</v>
+        <v>26.06564217464059</v>
       </c>
       <c r="D42" t="n">
-        <v>-17.25558377923974</v>
+        <v>3.156462640562879</v>
       </c>
       <c r="E42" t="s">
         <v>17</v>
       </c>
       <c r="F42" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -1489,16 +1535,16 @@
         <v>41</v>
       </c>
       <c r="C43" t="n">
-        <v>11.0538195331335</v>
+        <v>17.23406299489677</v>
       </c>
       <c r="D43" t="n">
-        <v>-13.63172191462643</v>
+        <v>-18.71534302127812</v>
       </c>
       <c r="E43" t="s">
         <v>17</v>
       </c>
       <c r="F43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -1509,15 +1555,315 @@
         <v>42</v>
       </c>
       <c r="C44" t="n">
-        <v>-2.066511104759158</v>
+        <v>-15.23674654061881</v>
       </c>
       <c r="D44" t="n">
-        <v>24.54768424160156</v>
+        <v>-15.21640986076447</v>
       </c>
       <c r="E44" t="s">
         <v>17</v>
       </c>
       <c r="F44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" t="n">
+        <v>-4.229400398706723</v>
+      </c>
+      <c r="D45" t="n">
+        <v>12.59799188807671</v>
+      </c>
+      <c r="E45" t="s">
+        <v>17</v>
+      </c>
+      <c r="F45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" t="n">
+        <v>44</v>
+      </c>
+      <c r="C46" t="n">
+        <v>-7.585525158281533</v>
+      </c>
+      <c r="D46" t="n">
+        <v>-11.14638854582135</v>
+      </c>
+      <c r="E46" t="s">
+        <v>17</v>
+      </c>
+      <c r="F46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6">
+      <c r="A47" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" t="n">
+        <v>45</v>
+      </c>
+      <c r="C47" t="n">
+        <v>6.936342233167339</v>
+      </c>
+      <c r="D47" t="n">
+        <v>30.45356584416535</v>
+      </c>
+      <c r="E47" t="s">
+        <v>17</v>
+      </c>
+      <c r="F47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6">
+      <c r="A48" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" t="n">
+        <v>46</v>
+      </c>
+      <c r="C48" t="n">
+        <v>-27.36270515855208</v>
+      </c>
+      <c r="D48" t="n">
+        <v>3.820391673025171</v>
+      </c>
+      <c r="E48" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6">
+      <c r="A49" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" t="n">
+        <v>47</v>
+      </c>
+      <c r="C49" t="n">
+        <v>12.21262988442415</v>
+      </c>
+      <c r="D49" t="n">
+        <v>14.33645310392244</v>
+      </c>
+      <c r="E49" t="s">
+        <v>17</v>
+      </c>
+      <c r="F49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" t="n">
+        <v>48</v>
+      </c>
+      <c r="C50" t="n">
+        <v>-3.039800158258757</v>
+      </c>
+      <c r="D50" t="n">
+        <v>11.3299682663736</v>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+      <c r="F50" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" t="n">
+        <v>49</v>
+      </c>
+      <c r="C51" t="n">
+        <v>-22.38024991159007</v>
+      </c>
+      <c r="D51" t="n">
+        <v>-8.290482612828129</v>
+      </c>
+      <c r="E51" t="s">
+        <v>17</v>
+      </c>
+      <c r="F51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" t="n">
+        <v>50</v>
+      </c>
+      <c r="C52" t="n">
+        <v>-14.7553421001751</v>
+      </c>
+      <c r="D52" t="n">
+        <v>21.73706300018365</v>
+      </c>
+      <c r="E52" t="s">
+        <v>17</v>
+      </c>
+      <c r="F52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" t="n">
+        <v>51</v>
+      </c>
+      <c r="C53" t="n">
+        <v>14.09060319255523</v>
+      </c>
+      <c r="D53" t="n">
+        <v>8.945564849255105</v>
+      </c>
+      <c r="E53" t="s">
+        <v>17</v>
+      </c>
+      <c r="F53" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B54" t="n">
+        <v>52</v>
+      </c>
+      <c r="C54" t="n">
+        <v>-6.06715556140871</v>
+      </c>
+      <c r="D54" t="n">
+        <v>18.08121041562056</v>
+      </c>
+      <c r="E54" t="s">
+        <v>17</v>
+      </c>
+      <c r="F54" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" t="n">
+        <v>53</v>
+      </c>
+      <c r="C55" t="n">
+        <v>14.28903032719646</v>
+      </c>
+      <c r="D55" t="n">
+        <v>-20.46054638787901</v>
+      </c>
+      <c r="E55" t="s">
+        <v>17</v>
+      </c>
+      <c r="F55" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6">
+      <c r="A56" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" t="n">
+        <v>54</v>
+      </c>
+      <c r="C56" t="n">
+        <v>10.40118487897376</v>
+      </c>
+      <c r="D56" t="n">
+        <v>-4.490369908150996</v>
+      </c>
+      <c r="E56" t="s">
+        <v>17</v>
+      </c>
+      <c r="F56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6">
+      <c r="A57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B57" t="n">
+        <v>55</v>
+      </c>
+      <c r="C57" t="n">
+        <v>-1.763308357209354</v>
+      </c>
+      <c r="D57" t="n">
+        <v>7.087722916941972</v>
+      </c>
+      <c r="E57" t="s">
+        <v>17</v>
+      </c>
+      <c r="F57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6">
+      <c r="A58" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B58" t="n">
+        <v>56</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.318304742319043</v>
+      </c>
+      <c r="D58" t="n">
+        <v>-2.198897941952368</v>
+      </c>
+      <c r="E58" t="s">
+        <v>17</v>
+      </c>
+      <c r="F58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6">
+      <c r="A59" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B59" t="n">
+        <v>57</v>
+      </c>
+      <c r="C59" t="n">
+        <v>-8.177937969688578</v>
+      </c>
+      <c r="D59" t="n">
+        <v>-21.85798934431147</v>
+      </c>
+      <c r="E59" t="s">
+        <v>17</v>
+      </c>
+      <c r="F59" t="b">
         <v>0</v>
       </c>
     </row>
@@ -1532,755 +1878,656 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:C59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>75</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="1" t="n">
+      <c r="B2" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="D2" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>23.94865099677753</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+      <c r="C2" t="n">
+        <v>2.145783012867295</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="n">
-        <v>16.82869086366553</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+      <c r="B3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>26.24499798705829</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="1" t="n">
+      <c r="B4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" t="n">
-        <v>17.21073956844748</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+      <c r="C4" t="n">
+        <v>11.3297339723723</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="1" t="n">
+      <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" t="n">
-        <v>9.263062716667703</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+      <c r="C5" t="n">
+        <v>33.60200418543344</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="1" t="n">
+      <c r="B6" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" t="n">
-        <v>20.98672650836765</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="C6" t="n">
+        <v>23.61158847221721</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="1" t="n">
+      <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D7" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="E7" t="n">
-        <v>21.70851647633481</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="C7" t="n">
+        <v>30.05940074136868</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="1" t="n">
+      <c r="B8" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D8" s="1" t="n">
-        <v>6</v>
-      </c>
-      <c r="E8" t="n">
-        <v>6.201568913875604</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5">
+      <c r="C8" t="n">
+        <v>30.62284658747639</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="1" t="n">
+      <c r="B9" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="1" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" t="n">
-        <v>22.9240927552754</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
+      <c r="C9" t="n">
+        <v>26.93047520653213</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10" s="1" t="n">
+      <c r="B10" s="1" t="n">
         <v>8</v>
       </c>
-      <c r="D10" s="1" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" t="n">
-        <v>21.27318504755872</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+      <c r="C10" t="n">
+        <v>23.23343656808299</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="1" t="n">
+      <c r="B11" s="1" t="n">
         <v>9</v>
       </c>
-      <c r="D11" s="1" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" t="n">
-        <v>4.956646536978488</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5">
+      <c r="C11" t="n">
+        <v>29.40932511489485</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C12" s="1" t="n">
+      <c r="B12" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D12" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="E12" t="n">
-        <v>16.99760439380548</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
+      <c r="C12" t="n">
+        <v>9.325313624883758</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="1" t="n">
+      <c r="B13" s="1" t="n">
         <v>11</v>
       </c>
-      <c r="D13" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="E13" t="n">
-        <v>15.87532706620174</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
+      <c r="C13" t="n">
+        <v>6.962327857642332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="1" t="n">
+      <c r="B14" s="1" t="n">
         <v>12</v>
       </c>
-      <c r="D14" s="1" t="n">
-        <v>12</v>
-      </c>
-      <c r="E14" t="n">
-        <v>20.27134275272189</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+      <c r="C14" t="n">
+        <v>20.61503469974378</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C15" s="1" t="n">
+      <c r="B15" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="D15" s="1" t="n">
-        <v>13</v>
-      </c>
-      <c r="E15" t="n">
-        <v>23.21361779150942</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+      <c r="C15" t="n">
+        <v>35.30718275687315</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="1" t="n">
+      <c r="B16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="D16" s="1" t="n">
-        <v>14</v>
-      </c>
-      <c r="E16" t="n">
-        <v>7.818772844355987</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+      <c r="C16" t="n">
+        <v>29.73430230241554</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C17" s="1" t="n">
+      <c r="B17" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="D17" s="1" t="n">
-        <v>15</v>
-      </c>
-      <c r="E17" t="n">
-        <v>22.53129303438007</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5">
+      <c r="C17" t="n">
+        <v>21.33400885121691</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="1" t="n">
+      <c r="B18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="D18" s="1" t="n">
-        <v>16</v>
-      </c>
-      <c r="E18" t="n">
-        <v>11.86554327508658</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5">
+      <c r="C18" t="n">
+        <v>26.32306066491322</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="D19" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="E19" t="n">
-        <v>21.82378786620968</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5">
+      <c r="B19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="C19" t="n">
+        <v>8.177566208936263</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C20" s="1" t="n">
+      <c r="B20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="D20" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="E20" t="n">
-        <v>12.14950470410536</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5">
+      <c r="C20" t="n">
+        <v>21.15690245477524</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C21" s="1" t="n">
+      <c r="B21" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="D21" s="1" t="n">
-        <v>19</v>
-      </c>
-      <c r="E21" t="n">
-        <v>29.74596566889847</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5">
+      <c r="C21" t="n">
+        <v>27.54423155893729</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="1" t="n">
+      <c r="B22" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="D22" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="E22" t="n">
-        <v>28.48358837045081</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
+      <c r="C22" t="n">
+        <v>20.15856758020352</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="1" t="n">
+      <c r="B23" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="D23" s="1" t="n">
-        <v>21</v>
-      </c>
-      <c r="E23" t="n">
-        <v>21.10245222493083</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5">
+      <c r="C23" t="n">
+        <v>27.21659702087382</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="1" t="n">
+      <c r="B24" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="D24" s="1" t="n">
-        <v>22</v>
-      </c>
-      <c r="E24" t="n">
-        <v>13.35169591707897</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5">
+      <c r="C24" t="n">
+        <v>12.6025429531584</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C25" s="1" t="n">
+      <c r="B25" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="D25" s="1" t="n">
-        <v>23</v>
-      </c>
-      <c r="E25" t="n">
-        <v>18.51518991923844</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5">
+      <c r="C25" t="n">
+        <v>18.98484567362867</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="1" t="n">
+      <c r="B26" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="D26" s="1" t="n">
-        <v>24</v>
-      </c>
-      <c r="E26" t="n">
-        <v>17.63865728521221</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5">
+      <c r="C26" t="n">
+        <v>18.59573177768589</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C27" s="1" t="n">
+      <c r="B27" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="D27" s="1" t="n">
-        <v>25</v>
-      </c>
-      <c r="E27" t="n">
-        <v>8.672837360440294</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5">
+      <c r="C27" t="n">
+        <v>22.65658416648923</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C28" s="1" t="n">
+      <c r="B28" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="D28" s="1" t="n">
-        <v>26</v>
-      </c>
-      <c r="E28" t="n">
-        <v>11.17996514380557</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
+      <c r="C28" t="n">
+        <v>30.55345411926473</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C29" s="1" t="n">
+      <c r="B29" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="D29" s="1" t="n">
-        <v>27</v>
-      </c>
-      <c r="E29" t="n">
-        <v>16.38884115579032</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5">
+      <c r="C29" t="n">
+        <v>28.35925320694647</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="1" t="n">
+      <c r="B30" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="D30" s="1" t="n">
-        <v>28</v>
-      </c>
-      <c r="E30" t="n">
-        <v>9.715783933962321</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5">
+      <c r="C30" t="n">
+        <v>0.5163230963155445</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="1" t="n">
+      <c r="B31" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="D31" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="E31" t="n">
-        <v>14.0727867442805</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5">
+      <c r="C31" t="n">
+        <v>12.51002737892676</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C32" s="1" t="n">
+      <c r="B32" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="D32" s="1" t="n">
-        <v>30</v>
-      </c>
-      <c r="E32" t="n">
-        <v>10.70225566226142</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="C32" t="n">
+        <v>9.592739365266546</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
       <c r="A33" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C33" s="1" t="n">
+      <c r="B33" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="D33" s="1" t="n">
-        <v>31</v>
-      </c>
-      <c r="E33" t="n">
-        <v>13.60069921258569</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="C33" t="n">
+        <v>5.644784122469007</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" s="1" t="n">
+      <c r="B34" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="D34" s="1" t="n">
-        <v>32</v>
-      </c>
-      <c r="E34" t="n">
-        <v>25.73617123929208</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="C34" t="n">
+        <v>21.59693977205388</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
       <c r="A35" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B35" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C35" s="1" t="n">
+      <c r="B35" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="D35" s="1" t="n">
-        <v>33</v>
-      </c>
-      <c r="E35" t="n">
-        <v>13.9392281146264</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="C35" t="n">
+        <v>16.99836392869713</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B36" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C36" s="1" t="n">
+      <c r="B36" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="D36" s="1" t="n">
-        <v>34</v>
-      </c>
-      <c r="E36" t="n">
-        <v>17.32206093675309</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="C36" t="n">
+        <v>14.9586881689375</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B37" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C37" s="1" t="n">
+      <c r="B37" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="D37" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="E37" t="n">
-        <v>17.77995294400602</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="C37" t="n">
+        <v>14.23136905153202</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B38" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C38" s="1" t="n">
+      <c r="B38" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="D38" s="1" t="n">
-        <v>36</v>
-      </c>
-      <c r="E38" t="n">
-        <v>24.7927828253155</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="C38" t="n">
+        <v>19.24148756668894</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B39" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="1" t="n">
+      <c r="B39" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="D39" s="1" t="n">
-        <v>37</v>
-      </c>
-      <c r="E39" t="n">
-        <v>14.47227201195521</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="C39" t="n">
+        <v>25.70302387727502</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="1" t="n">
+      <c r="B40" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="D40" s="1" t="n">
-        <v>38</v>
-      </c>
-      <c r="E40" t="n">
-        <v>22.44277302469148</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="C40" t="n">
+        <v>28.96433826167509</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C41" s="1" t="n">
+      <c r="B41" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="D41" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="E41" t="n">
-        <v>9.85452438844805</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="C41" t="n">
+        <v>16.89058784848077</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B42" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C42" s="1" t="n">
+      <c r="B42" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="D42" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="E42" t="n">
-        <v>20.83286703553734</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5">
+      <c r="C42" t="n">
+        <v>26.55830513266619</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3">
       <c r="A43" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B43" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C43" s="1" t="n">
+      <c r="B43" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="D43" s="1" t="n">
-        <v>41</v>
-      </c>
-      <c r="E43" t="n">
-        <v>18.65798726313595</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5">
+      <c r="C43" t="n">
+        <v>24.10282033731087</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3">
       <c r="A44" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B44" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C44" s="1" t="n">
+      <c r="B44" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="D44" s="1" t="n">
-        <v>42</v>
-      </c>
-      <c r="E44" t="n">
-        <v>23.987259613998</v>
+      <c r="C44" t="n">
+        <v>23.04512706241528</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3">
+      <c r="A45" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B45" s="1" t="n">
+        <v>43</v>
+      </c>
+      <c r="C45" t="n">
+        <v>13.01920971413401</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3">
+      <c r="A46" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B46" s="1" t="n">
+        <v>44</v>
+      </c>
+      <c r="C46" t="n">
+        <v>13.94611407327717</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3">
+      <c r="A47" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B47" s="1" t="n">
+        <v>45</v>
+      </c>
+      <c r="C47" t="n">
+        <v>30.50067662057578</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3">
+      <c r="A48" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="1" t="n">
+        <v>46</v>
+      </c>
+      <c r="C48" t="n">
+        <v>25.30611127848498</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3">
+      <c r="A49" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B49" s="1" t="n">
+        <v>47</v>
+      </c>
+      <c r="C49" t="n">
+        <v>17.8705885412703</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3">
+      <c r="A50" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B50" s="1" t="n">
+        <v>48</v>
+      </c>
+      <c r="C50" t="n">
+        <v>10.53955641694504</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3">
+      <c r="A51" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B51" s="1" t="n">
+        <v>49</v>
+      </c>
+      <c r="C51" t="n">
+        <v>24.21779708941035</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3">
+      <c r="A52" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="C52" t="n">
+        <v>27.71241254236175</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3">
+      <c r="A53" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53" s="1" t="n">
+        <v>51</v>
+      </c>
+      <c r="C53" t="n">
+        <v>17.92754175575471</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B54" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="C54" t="n">
+        <v>19.85064731528694</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B55" s="1" t="n">
+        <v>53</v>
+      </c>
+      <c r="C55" t="n">
+        <v>24.28244070015385</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" s="1" t="n">
+        <v>54</v>
+      </c>
+      <c r="C56" t="n">
+        <v>12.74085632351055</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3">
+      <c r="A57" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B57" s="1" t="n">
+        <v>55</v>
+      </c>
+      <c r="C57" t="n">
+        <v>8.315943902467318</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3">
+      <c r="A58" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B58" s="1" t="n">
+        <v>56</v>
+      </c>
+      <c r="C58" t="n">
+        <v>0.4583320779332982</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3">
+      <c r="A59" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B59" s="1" t="n">
+        <v>57</v>
+      </c>
+      <c r="C59" t="n">
+        <v>23.56727048122157</v>
       </c>
     </row>
   </sheetData>
@@ -2299,13 +2546,13 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:3">

</xml_diff>